<commit_message>
Update to Sinop data
</commit_message>
<xml_diff>
--- a/rice_prices_data_clean.xlsx
+++ b/rice_prices_data_clean.xlsx
@@ -19649,9 +19649,7 @@
       <c r="L290" t="n">
         <v>5.9</v>
       </c>
-      <c r="M290" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="M290"/>
       <c r="N290" t="s">
         <v>35</v>
       </c>
@@ -19659,9 +19657,7 @@
       <c r="P290" t="s">
         <v>30</v>
       </c>
-      <c r="Q290" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="Q290"/>
       <c r="R290" t="n">
         <v>82.29354347826</v>
       </c>
@@ -19674,11 +19670,9 @@
       <c r="U290" t="n">
         <v>1.18451144358493</v>
       </c>
-      <c r="V290" t="n">
-        <v>1.18451144358493</v>
-      </c>
+      <c r="V290"/>
       <c r="W290" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="291">
@@ -19716,9 +19710,7 @@
       <c r="L291" t="n">
         <v>5.35</v>
       </c>
-      <c r="M291" t="n">
-        <v>5.35</v>
-      </c>
+      <c r="M291"/>
       <c r="N291" t="s">
         <v>35</v>
       </c>
@@ -19726,9 +19718,7 @@
       <c r="P291" t="s">
         <v>30</v>
       </c>
-      <c r="Q291" t="n">
-        <v>5.35</v>
-      </c>
+      <c r="Q291"/>
       <c r="R291" t="n">
         <v>82.29354347826</v>
       </c>
@@ -19741,11 +19731,9 @@
       <c r="U291" t="n">
         <v>1.07409088528464</v>
       </c>
-      <c r="V291" t="n">
-        <v>1.07409088528464</v>
-      </c>
+      <c r="V291"/>
       <c r="W291" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="292">
@@ -19836,9 +19824,7 @@
       <c r="L293" t="n">
         <v>4.99</v>
       </c>
-      <c r="M293" t="n">
-        <v>4.99</v>
-      </c>
+      <c r="M293"/>
       <c r="N293" t="s">
         <v>35</v>
       </c>
@@ -19846,9 +19832,7 @@
       <c r="P293" t="s">
         <v>30</v>
       </c>
-      <c r="Q293" t="n">
-        <v>4.99</v>
-      </c>
+      <c r="Q293"/>
       <c r="R293" t="n">
         <v>82.23586363636</v>
       </c>
@@ -19861,11 +19845,9 @@
       <c r="U293" t="n">
         <v>1.02859123851546</v>
       </c>
-      <c r="V293" t="n">
-        <v>1.02859123851546</v>
-      </c>
+      <c r="V293"/>
       <c r="W293" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="294">
@@ -19903,9 +19885,7 @@
       <c r="L294" t="n">
         <v>5.1</v>
       </c>
-      <c r="M294" t="n">
-        <v>5.1</v>
-      </c>
+      <c r="M294"/>
       <c r="N294" t="s">
         <v>35</v>
       </c>
@@ -19913,9 +19893,7 @@
       <c r="P294" t="s">
         <v>30</v>
       </c>
-      <c r="Q294" t="n">
-        <v>5.1</v>
-      </c>
+      <c r="Q294"/>
       <c r="R294" t="n">
         <v>82.23586363636</v>
       </c>
@@ -19928,11 +19906,9 @@
       <c r="U294" t="n">
         <v>1.05126559447472</v>
       </c>
-      <c r="V294" t="n">
-        <v>1.05126559447472</v>
-      </c>
+      <c r="V294"/>
       <c r="W294" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="295">
@@ -19970,9 +19946,7 @@
       <c r="L295" t="n">
         <v>5.25</v>
       </c>
-      <c r="M295" t="n">
-        <v>5.25</v>
-      </c>
+      <c r="M295"/>
       <c r="N295" t="s">
         <v>35</v>
       </c>
@@ -19980,9 +19954,7 @@
       <c r="P295" t="s">
         <v>30</v>
       </c>
-      <c r="Q295" t="n">
-        <v>5.25</v>
-      </c>
+      <c r="Q295"/>
       <c r="R295" t="n">
         <v>82.23586363636</v>
       </c>
@@ -19995,11 +19967,9 @@
       <c r="U295" t="n">
         <v>1.0821851707828</v>
       </c>
-      <c r="V295" t="n">
-        <v>1.0821851707828</v>
-      </c>
+      <c r="V295"/>
       <c r="W295" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="296">
@@ -20037,9 +20007,7 @@
       <c r="L296" t="n">
         <v>5.19</v>
       </c>
-      <c r="M296" t="n">
-        <v>5.19</v>
-      </c>
+      <c r="M296"/>
       <c r="N296" t="s">
         <v>35</v>
       </c>
@@ -20047,9 +20015,7 @@
       <c r="P296" t="s">
         <v>30</v>
       </c>
-      <c r="Q296" t="n">
-        <v>5.19</v>
-      </c>
+      <c r="Q296"/>
       <c r="R296" t="n">
         <v>82.23586363636</v>
       </c>
@@ -20062,11 +20028,9 @@
       <c r="U296" t="n">
         <v>1.06981734025957</v>
       </c>
-      <c r="V296" t="n">
-        <v>1.06981734025957</v>
-      </c>
+      <c r="V296"/>
       <c r="W296" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="297">

</xml_diff>